<commit_message>
Normalise Ltd Vatinterface flat-rate column to each row's own month
The Ltd template's M column ("Flat rate Scheme Applied") referenced a
scattered set of Sales month tabs (rows 8-16 read Sep, May, Mar, Jun,
Nov, Aug, Aug, Nov, Jun). Point rows 6-17 at their own month's G4,
matching the SE template's pattern, and extend the month-mapping
regression test to cover the M column.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012mDxaoTv97DNa41DXrsLWu
</commit_message>
<xml_diff>
--- a/app/templates/ltd/Vatreturns.xlsx
+++ b/app/templates/ltd/Vatreturns.xlsx
@@ -16405,7 +16405,7 @@
       </c>
       <c r="L8" s="115"/>
       <c r="M8" s="116">
-        <f>IF([2]Sep!$G$4&gt;0,[2]Sep!$G$4,0)</f>
+        <f>IF([2]Jun!$G$4&gt;0,[2]Jun!$G$4,0)</f>
         <v>0</v>
       </c>
       <c r="N8" s="57"/>
@@ -16454,7 +16454,7 @@
       </c>
       <c r="L9" s="115"/>
       <c r="M9" s="116">
-        <f>IF([2]May!$G$4&gt;0,[2]May!$G$4,0)</f>
+        <f>IF([2]Jul!$G$4&gt;0,[2]Jul!$G$4,0)</f>
         <v>0</v>
       </c>
       <c r="N9" s="57"/>
@@ -16503,7 +16503,7 @@
       </c>
       <c r="L10" s="115"/>
       <c r="M10" s="116">
-        <f>IF([2]Mar!$G$4&gt;0,[2]Mar!$G$4,0)</f>
+        <f>IF([2]Aug!$G$4&gt;0,[2]Aug!$G$4,0)</f>
         <v>0</v>
       </c>
       <c r="N10" s="57"/>
@@ -16552,7 +16552,7 @@
       </c>
       <c r="L11" s="115"/>
       <c r="M11" s="116">
-        <f>IF([2]Jun!$G$4&gt;0,[2]Jun!$G$4,0)</f>
+        <f>IF([2]Sep!$G$4&gt;0,[2]Sep!$G$4,0)</f>
         <v>0</v>
       </c>
       <c r="N11" s="57"/>
@@ -16601,7 +16601,7 @@
       </c>
       <c r="L12" s="115"/>
       <c r="M12" s="116">
-        <f>IF([2]Nov!$G$4&gt;0,[2]Nov!$G$4,0)</f>
+        <f>IF([2]Oct!$G$4&gt;0,[2]Oct!$G$4,0)</f>
         <v>0</v>
       </c>
       <c r="N12" s="57"/>
@@ -16650,7 +16650,7 @@
       </c>
       <c r="L13" s="115"/>
       <c r="M13" s="116">
-        <f>IF([2]Aug!$G$4&gt;0,[2]Aug!$G$4,0)</f>
+        <f>IF([2]Nov!$G$4&gt;0,[2]Nov!$G$4,0)</f>
         <v>0</v>
       </c>
       <c r="N13" s="57"/>
@@ -16699,7 +16699,7 @@
       </c>
       <c r="L14" s="115"/>
       <c r="M14" s="116">
-        <f>IF([2]Aug!$G$4&gt;0,[2]Aug!$G$4,0)</f>
+        <f>IF([2]Dec!$G$4&gt;0,[2]Dec!$G$4,0)</f>
         <v>0</v>
       </c>
       <c r="N14" s="57"/>
@@ -16748,7 +16748,7 @@
       </c>
       <c r="L15" s="115"/>
       <c r="M15" s="116">
-        <f>IF([2]Nov!$G$4&gt;0,[2]Nov!$G$4,0)</f>
+        <f>IF([2]Jan!$G$4&gt;0,[2]Jan!$G$4,0)</f>
         <v>0</v>
       </c>
       <c r="N15" s="57"/>
@@ -16797,7 +16797,7 @@
       </c>
       <c r="L16" s="115"/>
       <c r="M16" s="116">
-        <f>IF([2]Jun!$G$4&gt;0,[2]Jun!$G$4,0)</f>
+        <f>IF([2]Feb!$G$4&gt;0,[2]Feb!$G$4,0)</f>
         <v>0</v>
       </c>
       <c r="N16" s="57"/>

</xml_diff>

<commit_message>
Give the VAT workbooks a fifth consecutive quarter
The Vatinterface carried sixteen periods, so the fifth return form could
only reach the same quarter the fourth already declared. Both workbooks now
carry a twentieth interface row fed by a new S06Y2/P06Y2 entry sheet pair,
and the period dropdown runs to K16.

Q5 moves from fourteen months past the book's first month to fifteen, so
every form is a quarter on from the one before it. The two overlap warnings
become checks that fail a run where any period reaches two returns.

The Ltd Admin sheet already held the new period end and payment due dates on
B38 and B40. The SE Admin date list stopped at the period end, so the payment
due date goes on B25 and the generator writes it.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/app/templates/ltd/Vatreturns.xlsx
+++ b/app/templates/ltd/Vatreturns.xlsx
@@ -23,10 +23,12 @@
     <sheet name="S03Y1" sheetId="26" r:id="rId8"/>
     <sheet name="S04Y2" sheetId="25" r:id="rId9"/>
     <sheet name="S05Y2" sheetId="24" r:id="rId10"/>
+    <sheet name="S06Y2" sheetId="28" r:id="rId22"/>
     <sheet name="P02Y1" sheetId="23" r:id="rId11"/>
     <sheet name="P03Y1" sheetId="22" r:id="rId12"/>
     <sheet name="P04Y2" sheetId="21" r:id="rId13"/>
     <sheet name="P05Y2" sheetId="27" r:id="rId14"/>
+    <sheet name="P06Y2" sheetId="29" r:id="rId23"/>
   </sheets>
   <externalReferences>
     <externalReference r:id="rId15"/>
@@ -1409,6 +1411,11 @@
             <v>46203</v>
           </cell>
         </row>
+        <row r="40">
+          <cell r="B40">
+            <v>46234</v>
+          </cell>
+        </row>
       </sheetData>
     </sheetDataSet>
   </externalBook>
@@ -2357,7 +2364,10 @@
       <c r="G16" s="25"/>
       <c r="H16" s="10"/>
       <c r="I16" s="13"/>
-      <c r="K16" s="70"/>
+      <c r="K16" s="69">
+        <f>Vatinterface!B20</f>
+        <v>46203</v>
+      </c>
     </row>
     <row r="17" spans="1:11" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A17" s="68"/>
@@ -2617,7 +2627,7 @@
   <phoneticPr fontId="5" type="noConversion"/>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G5" xr:uid="{839B348C-E01B-2843-A62A-D6136BF93408}">
-      <formula1>$K$2:$K$15</formula1>
+      <formula1>$K$2:$K$16</formula1>
     </dataValidation>
   </dataValidations>
   <printOptions horizontalCentered="1"/>
@@ -11560,6 +11570,4367 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
   <sheetPr codeName="Sheet14"/>
+  <dimension ref="A1:H201"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
+  <cols>
+    <col min="1" max="1" width="8.83203125" style="93" customWidth="1"/>
+    <col min="2" max="2" width="19.6640625" style="87" customWidth="1"/>
+    <col min="3" max="3" width="12.6640625" style="92" customWidth="1"/>
+    <col min="4" max="4" width="14.6640625" style="90" customWidth="1"/>
+    <col min="5" max="5" width="5.5" style="89" customWidth="1"/>
+    <col min="6" max="6" width="10.5" style="88" customWidth="1"/>
+    <col min="7" max="7" width="9.6640625" style="88" customWidth="1"/>
+    <col min="8" max="8" width="10.6640625" style="88" customWidth="1"/>
+    <col min="9" max="16384" width="9.1640625" style="87"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" s="75" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A1" s="150" t="s">
+        <v>36</v>
+      </c>
+      <c r="B1" s="151"/>
+      <c r="C1" s="169"/>
+      <c r="D1" s="163" t="s">
+        <v>29</v>
+      </c>
+      <c r="E1" s="164"/>
+      <c r="F1" s="86">
+        <f>SUM(F5:F200)</f>
+        <v>0</v>
+      </c>
+      <c r="G1" s="86">
+        <f>SUM(G5:G200)</f>
+        <v>0</v>
+      </c>
+      <c r="H1" s="86">
+        <f>SUM(H5:H200)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" s="102" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A2" s="166" t="s">
+        <v>35</v>
+      </c>
+      <c r="B2" s="160" t="str">
+        <f>IF((H1-SUM(O1:AK1)&lt;&gt;0),"COMPLETE EXPENSE ANALYSIS by inserting expense letter in col F","Supplier")</f>
+        <v>Supplier</v>
+      </c>
+      <c r="C2" s="170" t="s">
+        <v>34</v>
+      </c>
+      <c r="D2" s="148" t="s">
+        <v>33</v>
+      </c>
+      <c r="E2" s="165"/>
+      <c r="F2" s="160" t="s">
+        <v>32</v>
+      </c>
+      <c r="G2" s="103">
+        <f>[3]ClosingCreditors!$G$2</f>
+        <v>20</v>
+      </c>
+      <c r="H2" s="160" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" s="101" customFormat="1" ht="12" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A3" s="167"/>
+      <c r="B3" s="167"/>
+      <c r="C3" s="167"/>
+      <c r="D3" s="159"/>
+      <c r="E3" s="165"/>
+      <c r="F3" s="161"/>
+      <c r="G3" s="160" t="s">
+        <v>30</v>
+      </c>
+      <c r="H3" s="161"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A4" s="168"/>
+      <c r="B4" s="168"/>
+      <c r="C4" s="168"/>
+      <c r="D4" s="159"/>
+      <c r="E4" s="165"/>
+      <c r="F4" s="162"/>
+      <c r="G4" s="171"/>
+      <c r="H4" s="162"/>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="B5" s="89"/>
+      <c r="C5" s="91"/>
+      <c r="D5" s="89"/>
+      <c r="E5" s="87"/>
+      <c r="F5" s="100"/>
+      <c r="G5" s="88" t="str">
+        <f t="shared" ref="G5:G14" si="0">IF(F5&lt;&gt;0,F5*G$2/(100+G$2)," ")</f>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H5" s="88" t="str">
+        <f t="shared" ref="H5:H68" si="1">IF((F5&lt;&gt;0),F5-G5," ")</f>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="E6" s="87"/>
+      <c r="G6" s="88" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H6" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="E7" s="87"/>
+      <c r="G7" s="88" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H7" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="E8" s="87"/>
+      <c r="G8" s="88" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H8" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="E9" s="87"/>
+      <c r="G9" s="88" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H9" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="E10" s="87"/>
+      <c r="G10" s="88" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H10" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="E11" s="87"/>
+      <c r="G11" s="88" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H11" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="E12" s="87"/>
+      <c r="G12" s="88" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H12" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="E13" s="87"/>
+      <c r="G13" s="88" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H13" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="E14" s="87"/>
+      <c r="G14" s="88" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H14" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="E15" s="87"/>
+      <c r="G15" s="88" t="str">
+        <f t="shared" ref="G15:G78" si="2">IF(G$4="X"," ",IF(F15&lt;&gt;0,F15*G$2/(100+G$2)," "))</f>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H15" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="E16" s="87"/>
+      <c r="G16" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H16" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="17" spans="4:8" x14ac:dyDescent="0.15">
+      <c r="E17" s="87"/>
+      <c r="G17" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H17" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="18" spans="4:8" x14ac:dyDescent="0.15">
+      <c r="E18" s="87"/>
+      <c r="G18" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H18" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="19" spans="4:8" x14ac:dyDescent="0.15">
+      <c r="E19" s="87"/>
+      <c r="G19" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H19" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="20" spans="4:8" x14ac:dyDescent="0.15">
+      <c r="E20" s="87"/>
+      <c r="G20" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H20" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="21" spans="4:8" x14ac:dyDescent="0.15">
+      <c r="E21" s="87"/>
+      <c r="G21" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H21" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="22" spans="4:8" x14ac:dyDescent="0.15">
+      <c r="D22" s="87"/>
+      <c r="E22" s="87"/>
+      <c r="G22" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H22" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="23" spans="4:8" x14ac:dyDescent="0.15">
+      <c r="D23" s="99"/>
+      <c r="E23" s="87"/>
+      <c r="G23" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H23" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="24" spans="4:8" x14ac:dyDescent="0.15">
+      <c r="E24" s="87"/>
+      <c r="G24" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H24" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="25" spans="4:8" x14ac:dyDescent="0.15">
+      <c r="E25" s="87"/>
+      <c r="G25" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H25" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="26" spans="4:8" x14ac:dyDescent="0.15">
+      <c r="E26" s="87"/>
+      <c r="G26" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H26" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="27" spans="4:8" x14ac:dyDescent="0.15">
+      <c r="E27" s="87"/>
+      <c r="G27" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H27" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="28" spans="4:8" x14ac:dyDescent="0.15">
+      <c r="E28" s="87"/>
+      <c r="G28" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H28" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="29" spans="4:8" x14ac:dyDescent="0.15">
+      <c r="E29" s="87"/>
+      <c r="G29" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H29" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="30" spans="4:8" x14ac:dyDescent="0.15">
+      <c r="E30" s="87"/>
+      <c r="G30" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H30" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="31" spans="4:8" x14ac:dyDescent="0.15">
+      <c r="E31" s="87"/>
+      <c r="G31" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H31" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="32" spans="4:8" x14ac:dyDescent="0.15">
+      <c r="E32" s="87"/>
+      <c r="G32" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H32" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="33" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E33" s="87"/>
+      <c r="G33" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H33" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="34" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E34" s="87"/>
+      <c r="G34" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H34" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="35" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E35" s="87"/>
+      <c r="G35" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H35" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="36" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E36" s="87"/>
+      <c r="G36" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H36" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="37" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E37" s="87"/>
+      <c r="G37" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H37" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="38" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E38" s="87"/>
+      <c r="G38" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H38" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="39" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E39" s="87"/>
+      <c r="G39" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H39" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="40" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E40" s="87"/>
+      <c r="G40" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H40" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="41" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E41" s="87"/>
+      <c r="G41" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H41" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="42" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E42" s="87"/>
+      <c r="G42" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H42" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="43" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E43" s="87"/>
+      <c r="G43" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H43" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="44" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E44" s="87"/>
+      <c r="G44" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H44" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="45" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E45" s="87"/>
+      <c r="G45" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H45" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="46" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E46" s="87"/>
+      <c r="G46" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H46" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="47" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E47" s="87"/>
+      <c r="G47" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H47" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="48" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E48" s="87"/>
+      <c r="G48" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H48" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="49" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E49" s="87"/>
+      <c r="G49" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H49" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="50" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E50" s="87"/>
+      <c r="G50" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H50" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="51" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E51" s="87"/>
+      <c r="G51" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H51" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="52" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E52" s="87"/>
+      <c r="G52" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H52" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="53" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E53" s="87"/>
+      <c r="G53" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H53" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="54" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E54" s="87"/>
+      <c r="G54" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H54" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="55" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E55" s="87"/>
+      <c r="G55" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H55" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="56" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E56" s="87"/>
+      <c r="G56" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H56" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="57" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E57" s="87"/>
+      <c r="G57" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H57" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="58" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E58" s="87"/>
+      <c r="G58" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H58" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="59" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E59" s="87"/>
+      <c r="G59" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H59" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="60" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E60" s="87"/>
+      <c r="G60" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H60" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="61" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E61" s="87"/>
+      <c r="G61" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H61" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="62" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E62" s="87"/>
+      <c r="G62" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H62" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="63" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E63" s="87"/>
+      <c r="G63" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H63" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="64" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E64" s="87"/>
+      <c r="G64" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H64" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="65" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E65" s="87"/>
+      <c r="G65" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H65" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="66" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E66" s="87"/>
+      <c r="G66" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H66" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="67" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E67" s="87"/>
+      <c r="G67" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H67" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="68" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E68" s="87"/>
+      <c r="G68" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H68" s="88" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="69" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E69" s="87"/>
+      <c r="G69" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H69" s="88" t="str">
+        <f t="shared" ref="H69:H132" si="3">IF((F69&lt;&gt;0),F69-G69," ")</f>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="70" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E70" s="87"/>
+      <c r="G70" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H70" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="71" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E71" s="87"/>
+      <c r="G71" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H71" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="72" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E72" s="87"/>
+      <c r="G72" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H72" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="73" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E73" s="87"/>
+      <c r="G73" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H73" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="74" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E74" s="87"/>
+      <c r="G74" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H74" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="75" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E75" s="87"/>
+      <c r="G75" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H75" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="76" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E76" s="87"/>
+      <c r="G76" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H76" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="77" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E77" s="87"/>
+      <c r="G77" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H77" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="78" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E78" s="87"/>
+      <c r="G78" s="88" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H78" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="79" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E79" s="87"/>
+      <c r="G79" s="88" t="str">
+        <f t="shared" ref="G79:G142" si="4">IF(G$4="X"," ",IF(F79&lt;&gt;0,F79*G$2/(100+G$2)," "))</f>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H79" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="80" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E80" s="87"/>
+      <c r="G80" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H80" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="81" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E81" s="87"/>
+      <c r="G81" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H81" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="82" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E82" s="87"/>
+      <c r="G82" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H82" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="83" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E83" s="87"/>
+      <c r="G83" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H83" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="84" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E84" s="87"/>
+      <c r="G84" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H84" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="85" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E85" s="87"/>
+      <c r="G85" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H85" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="86" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E86" s="87"/>
+      <c r="G86" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H86" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="87" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E87" s="87"/>
+      <c r="G87" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H87" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="88" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E88" s="87"/>
+      <c r="G88" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H88" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="89" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E89" s="87"/>
+      <c r="G89" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H89" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="90" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E90" s="87"/>
+      <c r="G90" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H90" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="91" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E91" s="87"/>
+      <c r="G91" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H91" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="92" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E92" s="87"/>
+      <c r="G92" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H92" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="93" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E93" s="87"/>
+      <c r="G93" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H93" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="94" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E94" s="87"/>
+      <c r="G94" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H94" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="95" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E95" s="87"/>
+      <c r="G95" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H95" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="96" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E96" s="87"/>
+      <c r="G96" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H96" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="97" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E97" s="87"/>
+      <c r="G97" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H97" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="98" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E98" s="87"/>
+      <c r="G98" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H98" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="99" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E99" s="87"/>
+      <c r="G99" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H99" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="100" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E100" s="87"/>
+      <c r="G100" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H100" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="101" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E101" s="87"/>
+      <c r="G101" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H101" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="102" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E102" s="87"/>
+      <c r="G102" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H102" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="103" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E103" s="87"/>
+      <c r="G103" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H103" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="104" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E104" s="87"/>
+      <c r="G104" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H104" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="105" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E105" s="87"/>
+      <c r="G105" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H105" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="106" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E106" s="87"/>
+      <c r="G106" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H106" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="107" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E107" s="87"/>
+      <c r="G107" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H107" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="108" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E108" s="87"/>
+      <c r="G108" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H108" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="109" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E109" s="87"/>
+      <c r="G109" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H109" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="110" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E110" s="87"/>
+      <c r="G110" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H110" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="111" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E111" s="87"/>
+      <c r="G111" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H111" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="112" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E112" s="87"/>
+      <c r="G112" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H112" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="113" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E113" s="87"/>
+      <c r="G113" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H113" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="114" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E114" s="87"/>
+      <c r="G114" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H114" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="115" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E115" s="87"/>
+      <c r="G115" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H115" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="116" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E116" s="87"/>
+      <c r="G116" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H116" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="117" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E117" s="87"/>
+      <c r="G117" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H117" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="118" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E118" s="87"/>
+      <c r="G118" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H118" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="119" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E119" s="87"/>
+      <c r="G119" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H119" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="120" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E120" s="87"/>
+      <c r="G120" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H120" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="121" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E121" s="87"/>
+      <c r="G121" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H121" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="122" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E122" s="87"/>
+      <c r="G122" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H122" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="123" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E123" s="87"/>
+      <c r="G123" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H123" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="124" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E124" s="87"/>
+      <c r="G124" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H124" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="125" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E125" s="87"/>
+      <c r="G125" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H125" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="126" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E126" s="87"/>
+      <c r="G126" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H126" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="127" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E127" s="87"/>
+      <c r="G127" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H127" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="128" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E128" s="87"/>
+      <c r="G128" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H128" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="129" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E129" s="87"/>
+      <c r="G129" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H129" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="130" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E130" s="87"/>
+      <c r="G130" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H130" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="131" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E131" s="87"/>
+      <c r="G131" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H131" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="132" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E132" s="87"/>
+      <c r="G132" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H132" s="88" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="133" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E133" s="87"/>
+      <c r="G133" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H133" s="88" t="str">
+        <f t="shared" ref="H133:H196" si="5">IF((F133&lt;&gt;0),F133-G133," ")</f>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="134" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E134" s="87"/>
+      <c r="G134" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H134" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="135" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E135" s="87"/>
+      <c r="G135" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H135" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="136" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E136" s="87"/>
+      <c r="G136" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H136" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="137" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E137" s="87"/>
+      <c r="G137" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H137" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="138" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E138" s="87"/>
+      <c r="G138" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H138" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="139" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E139" s="87"/>
+      <c r="G139" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H139" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="140" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E140" s="87"/>
+      <c r="G140" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H140" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="141" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E141" s="87"/>
+      <c r="G141" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H141" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="142" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E142" s="87"/>
+      <c r="G142" s="88" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H142" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="143" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E143" s="87"/>
+      <c r="G143" s="88" t="str">
+        <f t="shared" ref="G143:G200" si="6">IF(G$4="X"," ",IF(F143&lt;&gt;0,F143*G$2/(100+G$2)," "))</f>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H143" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="144" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E144" s="87"/>
+      <c r="G144" s="88" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H144" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="145" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E145" s="87"/>
+      <c r="G145" s="88" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H145" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="146" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E146" s="87"/>
+      <c r="G146" s="88" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H146" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="147" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E147" s="87"/>
+      <c r="G147" s="88" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H147" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="148" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E148" s="87"/>
+      <c r="G148" s="88" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H148" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="149" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E149" s="87"/>
+      <c r="G149" s="88" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H149" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="150" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E150" s="87"/>
+      <c r="G150" s="88" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H150" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="151" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E151" s="87"/>
+      <c r="G151" s="88" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H151" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="152" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E152" s="87"/>
+      <c r="G152" s="88" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H152" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="153" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E153" s="87"/>
+      <c r="G153" s="88" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H153" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="154" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E154" s="87"/>
+      <c r="G154" s="88" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H154" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="155" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E155" s="87"/>
+      <c r="G155" s="88" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H155" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="156" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E156" s="87"/>
+      <c r="G156" s="88" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H156" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="157" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E157" s="87"/>
+      <c r="G157" s="88" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H157" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="158" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E158" s="87"/>
+      <c r="G158" s="88" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H158" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="159" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E159" s="87"/>
+      <c r="G159" s="88" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H159" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="160" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E160" s="87"/>
+      <c r="G160" s="88" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H160" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="161" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E161" s="87"/>
+      <c r="G161" s="88" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H161" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="162" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E162" s="87"/>
+      <c r="G162" s="88" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H162" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="163" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E163" s="87"/>
+      <c r="G163" s="88" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H163" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="164" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E164" s="87"/>
+      <c r="G164" s="88" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H164" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="165" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E165" s="87"/>
+      <c r="G165" s="88" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H165" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="166" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E166" s="87"/>
+      <c r="G166" s="88" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H166" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="167" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E167" s="87"/>
+      <c r="G167" s="88" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H167" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="168" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E168" s="87"/>
+      <c r="G168" s="88" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H168" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="169" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E169" s="87"/>
+      <c r="G169" s="88" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H169" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="170" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E170" s="87"/>
+      <c r="G170" s="88" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H170" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="171" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E171" s="87"/>
+      <c r="G171" s="88" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H171" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="172" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E172" s="87"/>
+      <c r="G172" s="88" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H172" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="173" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E173" s="87"/>
+      <c r="G173" s="88" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H173" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="174" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E174" s="87"/>
+      <c r="G174" s="88" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H174" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="175" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E175" s="87"/>
+      <c r="G175" s="88" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H175" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="176" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E176" s="87"/>
+      <c r="G176" s="88" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H176" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="177" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E177" s="87"/>
+      <c r="G177" s="88" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H177" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="178" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E178" s="87"/>
+      <c r="G178" s="88" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H178" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="179" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E179" s="87"/>
+      <c r="G179" s="88" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H179" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="180" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E180" s="87"/>
+      <c r="G180" s="88" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H180" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="181" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E181" s="87"/>
+      <c r="G181" s="88" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H181" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="182" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E182" s="87"/>
+      <c r="G182" s="88" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H182" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="183" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E183" s="87"/>
+      <c r="G183" s="88" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H183" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="184" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E184" s="87"/>
+      <c r="G184" s="88" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H184" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="185" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E185" s="87"/>
+      <c r="G185" s="88" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H185" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="186" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E186" s="87"/>
+      <c r="G186" s="88" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H186" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="187" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E187" s="87"/>
+      <c r="G187" s="88" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H187" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="188" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E188" s="87"/>
+      <c r="G188" s="88" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H188" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="189" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E189" s="87"/>
+      <c r="G189" s="88" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H189" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="190" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E190" s="87"/>
+      <c r="G190" s="88" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H190" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="191" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E191" s="87"/>
+      <c r="G191" s="88" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H191" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="192" spans="5:8" x14ac:dyDescent="0.15">
+      <c r="E192" s="87"/>
+      <c r="G192" s="88" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H192" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="193" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="E193" s="87"/>
+      <c r="G193" s="88" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H193" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="194" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="E194" s="87"/>
+      <c r="G194" s="88" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H194" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="195" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="E195" s="87"/>
+      <c r="G195" s="88" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H195" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="196" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="E196" s="87"/>
+      <c r="G196" s="88" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H196" s="88" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="197" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="E197" s="87"/>
+      <c r="G197" s="88" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H197" s="88" t="str">
+        <f>IF((F197&lt;&gt;0),F197-G197," ")</f>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="198" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="E198" s="87"/>
+      <c r="G198" s="88" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H198" s="88" t="str">
+        <f>IF((F198&lt;&gt;0),F198-G198," ")</f>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="199" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="E199" s="87"/>
+      <c r="G199" s="88" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H199" s="88" t="str">
+        <f>IF((F199&lt;&gt;0),F199-G199," ")</f>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="200" spans="1:8" ht="14" thickBot="1" x14ac:dyDescent="0.2">
+      <c r="A200" s="98"/>
+      <c r="B200" s="95"/>
+      <c r="C200" s="97"/>
+      <c r="D200" s="96"/>
+      <c r="E200" s="95"/>
+      <c r="F200" s="94"/>
+      <c r="G200" s="94" t="str">
+        <f t="shared" si="6"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H200" s="94" t="str">
+        <f>IF((F200&lt;&gt;0),F200-G200," ")</f>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="201" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A201" s="79" t="s">
+        <v>22</v>
+      </c>
+      <c r="G201" s="88" t="str">
+        <f>IF(F201&lt;&gt;0,F201*#REF!/(100+#REF!)," ")</f>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="10">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="A2:A4"/>
+    <mergeCell ref="B2:B4"/>
+    <mergeCell ref="H2:H4"/>
+    <mergeCell ref="G3:G4"/>
+    <mergeCell ref="D2:D4"/>
+    <mergeCell ref="F2:F4"/>
+    <mergeCell ref="E2:E4"/>
+    <mergeCell ref="C2:C4"/>
+  </mergeCells>
+  <phoneticPr fontId="5" type="noConversion"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter alignWithMargins="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
+  <sheetPr codeName="Sheet15"/>
+  <dimension ref="A1:H201"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
+  <cols>
+    <col min="1" max="1" width="9.1640625" style="79"/>
+    <col min="2" max="2" width="20.1640625" style="76" customWidth="1"/>
+    <col min="3" max="4" width="12.83203125" style="78" customWidth="1"/>
+    <col min="5" max="5" width="7.6640625" style="77" customWidth="1"/>
+    <col min="6" max="6" width="9.6640625" style="76" customWidth="1"/>
+    <col min="7" max="7" width="8.6640625" style="76" customWidth="1"/>
+    <col min="8" max="8" width="9.6640625" style="76" customWidth="1"/>
+    <col min="9" max="16384" width="9.1640625" style="75"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" s="85" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A1" s="150" t="s">
+        <v>36</v>
+      </c>
+      <c r="B1" s="151"/>
+      <c r="C1" s="152"/>
+      <c r="D1" s="153" t="s">
+        <v>29</v>
+      </c>
+      <c r="E1" s="154"/>
+      <c r="F1" s="86">
+        <f>SUM(F5:F500)</f>
+        <v>0</v>
+      </c>
+      <c r="G1" s="86">
+        <f>SUM(G5:G500)</f>
+        <v>0</v>
+      </c>
+      <c r="H1" s="86">
+        <f>SUM(H5:H500)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" s="85" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A2" s="146" t="s">
+        <v>28</v>
+      </c>
+      <c r="B2" s="144" t="s">
+        <v>27</v>
+      </c>
+      <c r="C2" s="149" t="s">
+        <v>26</v>
+      </c>
+      <c r="D2" s="155" t="s">
+        <v>39</v>
+      </c>
+      <c r="E2" s="158"/>
+      <c r="F2" s="144" t="s">
+        <v>25</v>
+      </c>
+      <c r="G2" s="121">
+        <f>[2]ClosingDebtors!$G$2</f>
+        <v>20</v>
+      </c>
+      <c r="H2" s="144" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" s="84" customFormat="1" ht="26" x14ac:dyDescent="0.15">
+      <c r="A3" s="147"/>
+      <c r="B3" s="148"/>
+      <c r="C3" s="149"/>
+      <c r="D3" s="156"/>
+      <c r="E3" s="158"/>
+      <c r="F3" s="144"/>
+      <c r="G3" s="120" t="s">
+        <v>23</v>
+      </c>
+      <c r="H3" s="144"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A4" s="145"/>
+      <c r="B4" s="145"/>
+      <c r="C4" s="145"/>
+      <c r="D4" s="157"/>
+      <c r="E4" s="159"/>
+      <c r="F4" s="145"/>
+      <c r="G4" s="122">
+        <f>[2]ClosingDebtors!$G$4</f>
+        <v>0</v>
+      </c>
+      <c r="H4" s="145"/>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="G5" s="76" t="str">
+        <f>IF(G$4&gt;0,(IF(F5&lt;&gt;0,F5*G$4/100," ")),IF(F5&lt;&gt;0,F5*G$2/(100+G$2)," "))</f>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H5" s="76" t="str">
+        <f t="shared" ref="H5:H68" si="0">IF((F5&lt;&gt;0),F5-G5," ")</f>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="G6" s="76" t="str">
+        <f t="shared" ref="G6:G69" si="1">IF(G$4&gt;0,(IF(F6&lt;&gt;0,F6*G$4/100," ")),IF(F6&lt;&gt;0,F6*G$2/(100+G$2)," "))</f>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H6" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="G7" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H7" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="G8" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H8" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="G9" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H9" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="G10" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H10" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="G11" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H11" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="G12" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H12" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="G13" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H13" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="G14" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H14" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="G15" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H15" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="G16" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H16" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="17" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G17" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H17" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="18" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G18" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H18" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="19" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G19" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H19" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="20" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G20" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H20" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="21" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G21" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H21" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="22" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G22" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H22" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="23" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G23" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H23" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="24" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G24" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H24" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="25" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G25" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H25" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="26" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G26" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H26" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="27" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G27" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H27" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="28" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G28" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H28" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="29" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G29" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H29" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="30" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G30" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H30" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="31" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G31" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H31" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="32" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G32" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H32" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="33" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G33" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H33" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="34" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G34" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H34" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="35" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G35" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H35" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="36" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G36" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H36" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="37" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G37" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H37" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="38" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G38" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H38" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="39" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G39" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H39" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="40" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G40" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H40" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="41" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G41" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H41" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="42" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G42" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H42" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="43" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G43" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H43" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="44" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G44" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H44" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="45" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G45" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H45" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="46" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G46" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H46" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="47" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G47" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H47" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="48" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G48" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H48" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="49" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G49" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H49" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="50" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G50" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H50" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="51" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G51" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H51" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="52" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G52" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H52" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="53" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G53" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H53" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="54" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G54" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H54" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="55" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G55" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H55" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="56" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G56" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H56" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="57" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G57" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H57" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="58" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G58" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H58" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="59" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G59" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H59" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="60" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G60" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H60" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="61" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G61" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H61" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="62" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G62" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H62" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="63" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G63" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H63" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="64" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G64" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H64" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="65" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G65" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H65" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="66" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G66" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H66" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="67" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G67" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H67" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="68" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G68" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H68" s="76" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="69" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G69" s="76" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H69" s="76" t="str">
+        <f t="shared" ref="H69:H132" si="2">IF((F69&lt;&gt;0),F69-G69," ")</f>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="70" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G70" s="76" t="str">
+        <f t="shared" ref="G70:G133" si="3">IF(G$4&gt;0,(IF(F70&lt;&gt;0,F70*G$4/100," ")),IF(F70&lt;&gt;0,F70*G$2/(100+G$2)," "))</f>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H70" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="71" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G71" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H71" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="72" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G72" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H72" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="73" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G73" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H73" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="74" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G74" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H74" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="75" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G75" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H75" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="76" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G76" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H76" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="77" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G77" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H77" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="78" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G78" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H78" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="79" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G79" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H79" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="80" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G80" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H80" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="81" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G81" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H81" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="82" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G82" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H82" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="83" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G83" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H83" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="84" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G84" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H84" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="85" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G85" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H85" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="86" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G86" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H86" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="87" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G87" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H87" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="88" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G88" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H88" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="89" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G89" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H89" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="90" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G90" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H90" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="91" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G91" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H91" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="92" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G92" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H92" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="93" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G93" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H93" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="94" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G94" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H94" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="95" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G95" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H95" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="96" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G96" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H96" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="97" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G97" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H97" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="98" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G98" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H98" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="99" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G99" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H99" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="100" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G100" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H100" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="101" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G101" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H101" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="102" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G102" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H102" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="103" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G103" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H103" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="104" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G104" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H104" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="105" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G105" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H105" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="106" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G106" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H106" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="107" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G107" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H107" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="108" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G108" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H108" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="109" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G109" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H109" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="110" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G110" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H110" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="111" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G111" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H111" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="112" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G112" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H112" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="113" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G113" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H113" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="114" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G114" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H114" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="115" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G115" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H115" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="116" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G116" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H116" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="117" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G117" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H117" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="118" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G118" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H118" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="119" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G119" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H119" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="120" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G120" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H120" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="121" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G121" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H121" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="122" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G122" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H122" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="123" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G123" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H123" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="124" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G124" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H124" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="125" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G125" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H125" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="126" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G126" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H126" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="127" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G127" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H127" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="128" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G128" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H128" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="129" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G129" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H129" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="130" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G130" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H130" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="131" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G131" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H131" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="132" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G132" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H132" s="76" t="str">
+        <f t="shared" si="2"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="133" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G133" s="76" t="str">
+        <f t="shared" si="3"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H133" s="76" t="str">
+        <f t="shared" ref="H133:H195" si="4">IF((F133&lt;&gt;0),F133-G133," ")</f>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="134" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G134" s="76" t="str">
+        <f t="shared" ref="G134:G197" si="5">IF(G$4&gt;0,(IF(F134&lt;&gt;0,F134*G$4/100," ")),IF(F134&lt;&gt;0,F134*G$2/(100+G$2)," "))</f>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H134" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="135" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G135" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H135" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="136" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G136" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H136" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="137" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G137" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H137" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="138" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G138" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H138" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="139" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G139" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H139" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="140" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G140" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H140" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="141" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G141" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H141" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="142" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G142" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H142" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="143" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G143" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H143" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="144" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G144" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H144" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="145" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G145" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H145" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="146" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G146" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H146" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="147" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G147" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H147" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="148" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G148" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H148" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="149" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G149" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H149" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="150" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G150" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H150" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="151" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G151" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H151" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="152" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G152" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H152" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="153" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G153" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H153" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="154" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G154" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H154" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="155" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G155" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H155" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="156" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G156" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H156" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="157" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G157" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H157" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="158" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G158" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H158" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="159" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G159" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H159" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="160" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G160" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H160" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="161" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G161" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H161" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="162" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G162" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H162" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="163" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G163" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H163" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="164" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G164" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H164" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="165" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G165" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H165" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="166" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G166" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H166" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="167" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G167" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H167" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="168" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G168" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H168" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="169" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G169" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H169" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="170" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G170" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H170" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="171" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G171" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H171" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="172" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G172" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H172" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="173" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G173" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H173" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="174" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G174" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H174" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="175" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G175" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H175" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="176" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G176" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H176" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="177" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G177" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H177" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="178" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G178" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H178" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="179" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G179" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H179" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="180" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G180" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H180" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="181" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G181" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H181" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="182" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G182" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H182" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="183" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G183" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H183" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="184" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G184" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H184" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="185" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G185" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H185" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="186" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G186" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H186" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="187" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G187" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H187" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="188" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G188" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H188" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="189" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G189" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H189" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="190" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G190" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H190" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="191" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G191" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H191" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="192" spans="7:8" x14ac:dyDescent="0.15">
+      <c r="G192" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H192" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="193" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="G193" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H193" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="194" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="G194" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H194" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="195" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="G195" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H195" s="76" t="str">
+        <f t="shared" si="4"/>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="196" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="G196" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H196" s="76" t="str">
+        <f>IF((F196&lt;&gt;0),F196-G196," ")</f>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="197" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="G197" s="76" t="str">
+        <f t="shared" si="5"/>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H197" s="76" t="str">
+        <f>IF((F197&lt;&gt;0),F197-G197," ")</f>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="198" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="G198" s="76" t="str">
+        <f>IF(G$4&gt;0,(IF(F198&lt;&gt;0,F198*G$4/100," ")),IF(F198&lt;&gt;0,F198*G$2/(100+G$2)," "))</f>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H198" s="76" t="str">
+        <f>IF((F198&lt;&gt;0),F198-G198," ")</f>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="199" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="G199" s="76" t="str">
+        <f>IF(G$4&gt;0,(IF(F199&lt;&gt;0,F199*G$4/100," ")),IF(F199&lt;&gt;0,F199*G$2/(100+G$2)," "))</f>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H199" s="76" t="str">
+        <f>IF((F199&lt;&gt;0),F199-G199," ")</f>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="200" spans="1:8" ht="14" thickBot="1" x14ac:dyDescent="0.2">
+      <c r="A200" s="83"/>
+      <c r="B200" s="80"/>
+      <c r="C200" s="82"/>
+      <c r="D200" s="82"/>
+      <c r="E200" s="81"/>
+      <c r="F200" s="80"/>
+      <c r="G200" s="80" t="str">
+        <f>IF(G$4&gt;0,(IF(F200&lt;&gt;0,F200*G$4/100," ")),IF(F200&lt;&gt;0,F200*G$2/(100+G$2)," "))</f>
+        <v xml:space="preserve"> </v>
+      </c>
+      <c r="H200" s="80" t="str">
+        <f>IF((F200&lt;&gt;0),F200-G200," ")</f>
+        <v xml:space="preserve"> </v>
+      </c>
+    </row>
+    <row r="201" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A201" s="79" t="s">
+        <v>22</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="H2:H4"/>
+    <mergeCell ref="A2:A4"/>
+    <mergeCell ref="B2:B4"/>
+    <mergeCell ref="C2:C4"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="D2:D4"/>
+    <mergeCell ref="E2:E4"/>
+    <mergeCell ref="F2:F4"/>
+  </mergeCells>
+  <phoneticPr fontId="5" type="noConversion"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter alignWithMargins="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0F00-000000000000}">
+  <sheetPr codeName="Sheet16"/>
   <dimension ref="A1:H201"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
@@ -14133,7 +18504,10 @@
       <c r="G16" s="25"/>
       <c r="H16" s="10"/>
       <c r="I16" s="13"/>
-      <c r="K16" s="70"/>
+      <c r="K16" s="69">
+        <f>Vatinterface!B20</f>
+        <v>46203</v>
+      </c>
     </row>
     <row r="17" spans="1:11" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A17" s="68"/>
@@ -14393,7 +18767,7 @@
   <phoneticPr fontId="5" type="noConversion"/>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G5" xr:uid="{00000000-0002-0000-0100-000000000000}">
-      <formula1>$K$2:$K$15</formula1>
+      <formula1>$K$2:$K$16</formula1>
     </dataValidation>
   </dataValidations>
   <printOptions horizontalCentered="1"/>
@@ -14699,7 +19073,10 @@
       <c r="G16" s="25"/>
       <c r="H16" s="10"/>
       <c r="I16" s="13"/>
-      <c r="K16" s="70"/>
+      <c r="K16" s="69">
+        <f>Vatinterface!B20</f>
+        <v>46203</v>
+      </c>
     </row>
     <row r="17" spans="1:11" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A17" s="68"/>
@@ -14959,7 +19336,7 @@
   <phoneticPr fontId="5" type="noConversion"/>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G5" xr:uid="{00000000-0002-0000-0200-000000000000}">
-      <formula1>$K$2:$K$15</formula1>
+      <formula1>$K$2:$K$16</formula1>
     </dataValidation>
   </dataValidations>
   <printOptions horizontalCentered="1"/>
@@ -15265,7 +19642,10 @@
       <c r="G16" s="25"/>
       <c r="H16" s="10"/>
       <c r="I16" s="13"/>
-      <c r="K16" s="70"/>
+      <c r="K16" s="69">
+        <f>Vatinterface!B20</f>
+        <v>46203</v>
+      </c>
     </row>
     <row r="17" spans="1:11" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A17" s="68"/>
@@ -15525,7 +19905,7 @@
   <phoneticPr fontId="5" type="noConversion"/>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G5" xr:uid="{00000000-0002-0000-0300-000000000000}">
-      <formula1>$K$2:$K$15</formula1>
+      <formula1>$K$2:$K$16</formula1>
     </dataValidation>
   </dataValidations>
   <printOptions horizontalCentered="1"/>
@@ -15831,7 +20211,10 @@
       <c r="G16" s="25"/>
       <c r="H16" s="10"/>
       <c r="I16" s="13"/>
-      <c r="K16" s="70"/>
+      <c r="K16" s="69">
+        <f>Vatinterface!B20</f>
+        <v>46203</v>
+      </c>
     </row>
     <row r="17" spans="1:11" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
       <c r="A17" s="68"/>
@@ -16091,7 +20474,7 @@
   <phoneticPr fontId="5" type="noConversion"/>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G5" xr:uid="{00000000-0002-0000-0400-000000000000}">
-      <formula1>$K$2:$K$15</formula1>
+      <formula1>$K$2:$K$16</formula1>
     </dataValidation>
   </dataValidations>
   <printOptions horizontalCentered="1"/>
@@ -16107,7 +20490,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <sheetPr codeName="Sheet6"/>
-  <dimension ref="A1:N20"/>
+  <dimension ref="A1:N21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="12" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="2" style="44" customWidth="1"/>
@@ -16906,7 +21289,7 @@
         <f>[1]Admin!$B$36</f>
         <v>46173</v>
       </c>
-      <c r="C19" s="63">
+      <c r="C19" s="62">
         <f>[1]Admin!$B$38</f>
         <v>46203</v>
       </c>
@@ -16949,21 +21332,70 @@
       </c>
       <c r="N19" s="57"/>
     </row>
-    <row r="20" spans="1:14" ht="9" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="58"/>
-      <c r="B20" s="59"/>
-      <c r="C20" s="59"/>
-      <c r="D20" s="60"/>
-      <c r="E20" s="60"/>
-      <c r="F20" s="60"/>
-      <c r="G20" s="60"/>
-      <c r="H20" s="60"/>
-      <c r="I20" s="60"/>
-      <c r="J20" s="60"/>
-      <c r="K20" s="60"/>
-      <c r="L20" s="117"/>
-      <c r="M20" s="118"/>
-      <c r="N20" s="61"/>
+    <row r="20" spans="1:14" x14ac:dyDescent="0.15">
+      <c r="A20" s="56"/>
+      <c r="B20" s="62">
+        <f>[1]Admin!$B$38</f>
+        <v>46203</v>
+      </c>
+      <c r="C20" s="63">
+        <f>[1]Admin!$B$40</f>
+        <v>46234</v>
+      </c>
+      <c r="D20" s="104">
+        <f>S06Y2!$H$1</f>
+        <v>0</v>
+      </c>
+      <c r="E20" s="105">
+        <f>SUM(D18:D20)</f>
+        <v>0</v>
+      </c>
+      <c r="F20" s="105">
+        <f>S06Y2!$G$1</f>
+        <v>0</v>
+      </c>
+      <c r="G20" s="105">
+        <f>SUM(F18:F20)</f>
+        <v>0</v>
+      </c>
+      <c r="H20" s="105">
+        <f>P06Y2!$H$1</f>
+        <v>0</v>
+      </c>
+      <c r="I20" s="105">
+        <f>SUM(H18:H20)</f>
+        <v>0</v>
+      </c>
+      <c r="J20" s="105">
+        <f>P06Y2!$G$1</f>
+        <v>0</v>
+      </c>
+      <c r="K20" s="105">
+        <f>SUM(J18:J20)</f>
+        <v>0</v>
+      </c>
+      <c r="L20" s="115"/>
+      <c r="M20" s="116">
+        <f>IF([2]Mar!$G$4&gt;0,[2]Mar!$G$4,0)</f>
+        <v>0</v>
+      </c>
+      <c r="N20" s="57"/>
+    </row>
+    <row r="21" spans="1:14" ht="9" customHeight="1" thickBot="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="58"/>
+      <c r="B21" s="59"/>
+      <c r="C21" s="59"/>
+      <c r="D21" s="60"/>
+      <c r="E21" s="60"/>
+      <c r="F21" s="60"/>
+      <c r="G21" s="60"/>
+      <c r="H21" s="60"/>
+      <c r="I21" s="60"/>
+      <c r="J21" s="60"/>
+      <c r="K21" s="60"/>
+      <c r="L21" s="117"/>
+      <c r="M21" s="118"/>
+      <c r="N21" s="61"/>
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>

</xml_diff>

<commit_message>
T3: remove 12 divider-row stray cells with broken #REF! formulas
Repair row 201 leftovers: remove formulas that lost their rate references
(IF(G201<>0,G201*#REF!/(100+#REF!)," ") in se/Vat.xlsx and similar in Ltd
files). Each cell replaced with styled empty cell preserving style index.

Verified:
- 12 cells found and replaced (H201 on P02Y1/P03Y1/P04Y2/P05Y2/P06Y2 in
  se/Vat.xlsx with style 90; G201 on same sheets in ltd/Vatreturns.xlsx
  with style 88; G201 on OpeningCreditors/ClosingCreditors in
  ltd/Purchases.xlsx with style 20)
- 0 remaining #REF! in all three workbooks
- formula-presence-guard test: 1282 tests passed

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016fw7EguSoRDRfzuaKQWp8b
</commit_message>
<xml_diff>
--- a/app/templates/ltd/Vatreturns.xlsx
+++ b/app/templates/ltd/Vatreturns.xlsx
@@ -6977,10 +6977,7 @@
       <c r="A201" s="79" t="s">
         <v>22</v>
       </c>
-      <c r="G201" s="88" t="str">
-        <f>IF(F201&lt;&gt;0,F201*#REF!/(100+#REF!)," ")</f>
-        <v xml:space="preserve"> </v>
-      </c>
+      <c r="G201" s="88"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -9260,10 +9257,7 @@
       <c r="A201" s="79" t="s">
         <v>22</v>
       </c>
-      <c r="G201" s="88" t="str">
-        <f>IF(F201&lt;&gt;0,F201*#REF!/(100+#REF!)," ")</f>
-        <v xml:space="preserve"> </v>
-      </c>
+      <c r="G201" s="88"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -11543,10 +11537,7 @@
       <c r="A201" s="79" t="s">
         <v>22</v>
       </c>
-      <c r="G201" s="88" t="str">
-        <f>IF(F201&lt;&gt;0,F201*#REF!/(100+#REF!)," ")</f>
-        <v xml:space="preserve"> </v>
-      </c>
+      <c r="G201" s="88"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -13826,10 +13817,7 @@
       <c r="A201" s="79" t="s">
         <v>22</v>
       </c>
-      <c r="G201" s="88" t="str">
-        <f>IF(F201&lt;&gt;0,F201*#REF!/(100+#REF!)," ")</f>
-        <v xml:space="preserve"> </v>
-      </c>
+      <c r="G201" s="88"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -18187,10 +18175,7 @@
       <c r="A201" s="79" t="s">
         <v>22</v>
       </c>
-      <c r="G201" s="88" t="str">
-        <f>IF(F201&lt;&gt;0,F201*#REF!/(100+#REF!)," ")</f>
-        <v xml:space="preserve"> </v>
-      </c>
+      <c r="G201" s="88"/>
     </row>
   </sheetData>
   <mergeCells count="10">

</xml_diff>